<commit_message>
Templates: use supplied ISMS documents and policies, standard Document History
Replaces 18 templates with the supplied ISMS documents and policies (company names, personal
names and platform references removed, process content unchanged), adds the Management Review
and Corrective Action procedures, and gives every template the same Document History table
at the end of the document.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DQ8ZSi2UY9xjrq8oz1Heak
</commit_message>
<xml_diff>
--- a/netlify/template-files/acceptance-test-record.xlsx
+++ b/netlify/template-files/acceptance-test-record.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review and approval" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document History" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -492,95 +492,87 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>[x.x]</t>
+          <t>Records testing and acceptance of a release before production.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Document owner</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>[Role]</t>
+          <t>Each release.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Approver</t>
+          <t>Roles and responsibilities</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>[Role]</t>
+          <t>Engineering Lead: Owns the process.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Effective date</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>[YYYY-MM-DD]</t>
+          <t>Engineers: Follow it and record evidence.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Next review date</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>[YYYY-MM-DD]</t>
+          <t>Security Lead: Reviews periodically.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>1. List test cases run with results.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2. Record defects and their status.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
+      <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Records testing and acceptance of a release before production.</t>
+          <t>3. Product owner signs acceptance.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Frequency and timing</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -592,106 +584,38 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Roles and responsibilities</t>
+          <t>Audit evidence checklist</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Engineering Lead: Owns the process.</t>
+          <t>☐ Records for sampled releases</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Framework mapping</t>
+        </is>
+      </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Engineers: Follow it and record evidence.</t>
+          <t>ISO 27001: A.8.29</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Security Lead: Reviews periodically.</t>
-        </is>
-      </c>
+      <c r="B15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Procedure</t>
+          <t>Footer</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>1. List test cases run with results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>2. Record defects and their status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>3. Product owner signs acceptance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Frequency and timing</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Each release.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Audit evidence checklist</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>☐ Records for sampled releases</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Framework mapping</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>ISO 27001: A.8.29</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Footer</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Template provided by OneLens by Ruchi. Replace all [bracketed] fields before use.</t>
         </is>
@@ -1330,106 +1254,67 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Written by</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Approved by</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Prepared by</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Reviewed by</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Approved by</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Revision history</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Author</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Description of change</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>[YYYY-MM-DD]</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>[Role]</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Initial version</t>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>[TODAYS DATE]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Initial Version</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>[Name]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[Name]</t>
         </is>
       </c>
     </row>

</xml_diff>